<commit_message>
docs: record full name of Nguyen Bui Man Nhi
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -610,7 +610,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Cách điền: mỗi người tự chọn việc ở cột của mình (D–H), chọn "Chính" hoặc "Hỗ trợ" từ danh sách. Mỗi việc cần đúng một người "Chính". Cột Trạng thái chọn từ danh sách. Khung lập ngày 2026-09-17; họ tên Mẫn Nhi và Dương Khang chưa đầy đủ.</t>
+          <t>Cách điền: mỗi người tự chọn việc ở cột của mình (D–H), chọn "Chính" hoặc "Hỗ trợ" từ danh sách. Mỗi việc cần đúng một người "Chính". Cột Trạng thái chọn từ danh sách. Khung lập ngày 2026-09-17; họ tên Dương Khang chưa đầy đủ.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Mẫn Nhi
+          <t>Nguyễn Bùi Mẫn Nhi
 25C15055</t>
         </is>
       </c>

</xml_diff>

<commit_message>
docs: record full name of Au Duong Khang
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -610,7 +610,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Cách điền: mỗi người tự chọn việc ở cột của mình (D–H), chọn "Chính" hoặc "Hỗ trợ" từ danh sách. Mỗi việc cần đúng một người "Chính". Cột Trạng thái chọn từ danh sách. Khung lập ngày 2026-09-17; họ tên Dương Khang chưa đầy đủ.</t>
+          <t>Cách điền: mỗi người tự chọn việc ở cột của mình (D–H), chọn "Chính" hoặc "Hỗ trợ" từ danh sách. Mỗi việc cần đúng một người "Chính". Cột Trạng thái chọn từ danh sách. Khung lập ngày 2026-09-17.</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Dương Khang
+          <t>Âu Dương Khang
 25C15045</t>
         </is>
       </c>

</xml_diff>

<commit_message>
docs: Loc claims repo setup, CLIP features, data split and baseline tasks
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -682,14 +682,18 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n"/>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="7" t="n"/>
       <c r="G6" s="7" t="n"/>
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>
@@ -705,7 +709,11 @@
           <t>dùng chung</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n"/>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="n"/>
@@ -778,7 +786,11 @@
           <t>Visual Genome ∩ COCO</t>
         </is>
       </c>
-      <c r="D10" s="7" t="n"/>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="7" t="n"/>
       <c r="G10" s="7" t="n"/>
@@ -801,7 +813,11 @@
           <t>Visual Genome ∩ COCO</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n"/>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="E11" s="7" t="n"/>
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="7" t="n"/>
@@ -1453,6 +1469,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="C40" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: add end-to-end smoke test, record data checksums and setup instructions
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -693,7 +693,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       <c r="H7" s="7" t="n"/>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="C40" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: add CLIP feature extraction script for vg_coco, update task sheet
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -778,7 +778,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Dữ liệu: join theo coco_id, tập con cố định theo seed, split Karpathy, lưu file split</t>
+          <t>Dữ liệu: join theo coco_id, lấy toàn bộ phần giao (không lấy mẫu), split Karpathy, lưu file split</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -797,7 +797,7 @@
       <c r="H10" s="7" t="n"/>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1695,24 +1695,24 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Giữ ảnh có coco_id khác null. Gán split theo Karpathy (train / val / test). Lấy tập con theo seed cố định: đề xuất train 10 000, val 1 000, test 1 000 ảnh; mỗi ảnh 5 caption. Đếm và ghi lại: số ảnh giao, số ảnh mỗi split trước và sau khi lấy mẫu. Tải ảnh của tập con.</t>
+          <t>Giữ ảnh có coco_id khác null. Gán split theo Karpathy (restval gộp vào train). Lấy TOÀN BỘ phần giao, không lấy mẫu (chốt 2026-09-18): train 46 944, val 2 126, test 2 138 ảnh; 290 ảnh Visual Genome bị bỏ vì trùng coco_id. Tải ảnh bằng scripts/download_images.py (chỉ cần trên máy trích đặc trưng).</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>data/splits/vg_coco_train.json, _val.json, _test.json (image_id, coco_id, captions)
+          <t>data/splits/vg_coco_train.json, _val.json, _test.json
 data/raw/images/
 experiments/data_stats.md</t>
         </is>
       </c>
       <c r="F6" s="20" t="inlineStr">
         <is>
-          <t>src/data/build_split.py, pandas</t>
+          <t>src/data/build_split.py, scripts/download_images.py</t>
         </is>
       </c>
       <c r="G6" s="20" t="inlineStr">
         <is>
-          <t>Split lấy theo chuẩn có sẵn, không tự chia lại. Seed lấy mẫu ghi trong config. File split nộp kèm (Mục 6).</t>
+          <t>Split lấy theo chuẩn có sẵn, không tự chia lại và không lấy mẫu nên không phụ thuộc seed. File split nộp kèm (Mục 6).</t>
         </is>
       </c>
       <c r="H6" s="20" t="inlineStr">
@@ -2214,7 +2214,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="22" t="inlineStr">
         <is>
-          <t>1. Kích thước tập con (đề xuất 10 000 / 1 000 / 1 000 ảnh): chốt sau khi đếm số ảnh giao ở bước 1.2.</t>
+          <t>1. Kích thước tập con: ĐÃ CHỐT 2026-09-18, lấy toàn bộ phần giao (51 208 ảnh), không lấy mẫu.</t>
         </is>
       </c>
     </row>
@@ -2253,6 +2253,11 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A19:I19"/>

</xml_diff>

<commit_message>
docs: document the shared metrics module, update task sheet
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -736,14 +736,18 @@
           <t>dùng chung</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n"/>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="n"/>
       <c r="H8" s="7" t="n"/>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -797,7 +801,7 @@
       <c r="H10" s="7" t="n"/>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2253,11 +2257,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A19:I19"/>

</xml_diff>

<commit_message>
docs: mark Loc as support on the run instructions task
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -1462,7 +1462,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D38" s="7" t="n"/>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Hỗ trợ</t>
+        </is>
+      </c>
       <c r="E38" s="7" t="n"/>
       <c r="F38" s="7" t="n"/>
       <c r="G38" s="7" t="n"/>

</xml_diff>

<commit_message>
docs: switch level 1 graph design to per-image scene graphs
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -836,7 +836,7 @@
       <c r="A12" s="8" t="n"/>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Dựng đồ thị: lọc VG150, node ảnh + node khái niệm, cạnh chứa + quan hệ, cạnh ConceptNet</t>
+          <t>Dựng đồ thị: lọc VG150, mỗi ảnh một scene graph riêng (node đối tượng, cạnh quan hệ, bộ ba); thống kê đồ thị và đo tỉ lệ bộ ba của caption tìm thấy trong scene graph của ảnh gốc</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -859,7 +859,7 @@
       <c r="A13" s="8" t="n"/>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Nối truy vấn vào đồ thị: tách danh từ/động từ, khớp vào node khái niệm</t>
+          <t>Đồ thị truy vấn: tách caption thành bộ ba (chủ thể, quan hệ, đối tượng), chuẩn hoá tên theo alias VG150</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
@@ -882,7 +882,7 @@
       <c r="A14" s="8" t="n"/>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>GNN (GAT) và điểm đồ thị cho từng ứng viên trong top-k</t>
+          <t>GNN (GAT) chạy trong từng đồ thị nhỏ (ảnh và truy vấn); điểm đồ thị = độ khớp bộ ba cho từng ứng viên trong top-k</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
@@ -928,7 +928,7 @@
       <c r="A16" s="8" t="n"/>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Ablation: bỏ cạnh quan hệ, xáo cạnh, đồ thị ngẫu nhiên</t>
+          <t>Ablation: bỏ cạnh quan hệ (chỉ còn đối tượng), xáo cạnh trong scene graph, scene graph ngẫu nhiên</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -951,7 +951,7 @@
       <c r="A17" s="8" t="n"/>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Giải thích cơ bản: trích cạnh/đường đi đóng góp vào điểm đồ thị</t>
+          <t>Giải thích cơ bản: các cặp bộ ba khớp giữa truy vấn và ảnh, kèm đóng góp của từng cặp vào điểm đồ thị</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
@@ -1166,7 +1166,7 @@
       <c r="A26" s="9" t="n"/>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>Mở rộng (chọn 1–2): độ nhạy theo α, so các cách tạo cạnh</t>
+          <t>Mở rộng (chọn 1–2): độ nhạy theo α, so các cách tạo cạnh, lớp khái niệm ConceptNet cho truy vấn gián tiếp (bật/tắt là một ablation)</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -1561,7 +1561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1582,10 +1582,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Luồng: truy vấn (caption COCO) → CLIP → top-50 theo cosine → điểm đồ thị từ GAT trên scene graph + ConceptNet → xếp hạng lại → đường đi giải thích. Yêu cầu đề: so CLIP với CLIP + Graph trên cùng split, ablation bỏ/xáo cạnh, hiển thị đường đi, 5 thành công + 5 thất bại. Tên file là đề xuất, đổi được nhưng giữ tiếng Anh.</t>
+          <t>Luồng: truy vấn (caption COCO) → CLIP → top-50 theo cosine → tách truy vấn thành đồ thị nhỏ → GAT trên đồ thị truy vấn và trên scene graph của từng ảnh ứng viên → điểm đồ thị = độ khớp bộ ba → xếp hạng lại → giải thích bằng các bộ ba khớp. Mỗi ảnh một đồ thị riêng, KHÔNG dựng một đồ thị chung chứa mọi ảnh; ConceptNet để sang cấp độ 2 (đổi thiết kế 2026-09-19, xem ghi chú cuối sheet). Yêu cầu đề: so CLIP với CLIP + Graph trên cùng split, ablation bỏ/xáo cạnh, hiển thị đường đi, 5 thành công + 5 thất bại. Tên file là đề xuất, đổi được nhưng giữ tiếng Anh.</t>
         </is>
       </c>
     </row>
@@ -1747,17 +1747,17 @@
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>Ảnh tập con, caption, tên 150 lớp đối tượng.</t>
+          <t>Ảnh tập con, caption, nhãn VG150 (150 lớp đối tượng, 50 quan hệ).</t>
         </is>
       </c>
       <c r="D7" s="20" t="inlineStr">
         <is>
-          <t>open_clip, encoder đóng băng (bản nào thì chờ kết quả thử CLIP đa ngữ ở giai đoạn 0; mặc định ViT-B/32). Trích một lần: vector ảnh, vector caption, vector tên khái niệm theo mẫu "a photo of a {tên}". Chuẩn hoá L2.</t>
+          <t>open_clip, encoder đóng băng ViT-B/32 (openai). Trích một lần: vector ảnh, vector caption (đã xong), và vector nhãn VG150 để làm đặc trưng node/cạnh của đồ thị nhỏ (đối tượng theo mẫu "a photo of a {tên}", quan hệ mã hoá nguyên văn). Chuẩn hoá L2.</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
         <is>
-          <t>data/features/image_feats.npy, caption_feats.npy, concept_feats.npy + file ánh xạ id → dòng</t>
+          <t>data/features/vg_coco_image.npy, vg_coco_caption.npy, vg_coco_concept.npy + file .ids.json</t>
         </is>
       </c>
       <c r="F7" s="20" t="inlineStr">
@@ -1842,33 +1842,35 @@
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>objects.json, relationships.json, alias, danh sách VG150 (150 lớp đối tượng, 50 quan hệ), ConceptNet (assertions tiếng Anh).</t>
+          <t>objects.json, relationships.json, alias, danh sách VG150 (150 lớp đối tượng, 50 quan hệ), file split, caption.</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>Chuẩn hoá tên theo alias, lọc theo VG150. Node: ảnh + khái niệm. Cạnh: (ảnh, contains, khái niệm); (khái niệm, quan hệ, khái niệm) lấy từ scene graph; (khái niệm, RelatedTo / UsedFor / IsA / AtLocation / PartOf, khái niệm) lấy từ ConceptNet, có thể thêm node khái niệm ngoài VG150 nếu nó nối hai khái niệm VG150. Đặc trưng node: ảnh = vector CLIP ảnh, khái niệm = vector CLIP text.</t>
+          <t>Chuẩn hoá tên theo alias, lọc theo VG150. Mỗi ảnh một đồ thị riêng: node = đối tượng (nhãn VG150), cạnh có hướng = quan hệ, mỗi cạnh cho một bộ ba (chủ thể, quan hệ, đối tượng); gộp các đối tượng trùng nhãn chỉ khi trùng hộp bao. Đặc trưng node và cạnh = vector CLIP text của nhãn. Làm TRƯỚC khi viết GNN: script đo (a) số đối tượng / quan hệ mỗi ảnh sau lọc, tỉ lệ ảnh không còn quan hệ nào; (b) tỉ lệ caption tách ra được ≥1 bộ ba; (c) tỉ lệ bộ ba của caption tìm thấy trong scene graph của đúng ảnh gốc.</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>data/graphs/vg_coco_graph.pt (PyG HeteroData hoặc danh sách triple)
+          <t>data/graphs/vg_coco_scene_graphs.jsonl (mỗi dòng một ảnh)
+scripts/checks/scene_graph_coverage.py
+experiments/checks/scene_graph_coverage.json
 experiments/level1/graph_stats.md</t>
         </is>
       </c>
       <c r="F9" s="20" t="inlineStr">
         <is>
-          <t>src/graph/build_vg_graph.py, torch_geometric</t>
+          <t>src/graph/build_scene_graphs.py, torch_geometric</t>
         </is>
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>CHỖ DỄ RÒ RỈ NHẤT. Cạnh khái niệm–khái niệm gộp từ nhiều ảnh là cạnh thống kê → chỉ gộp từ ảnh TRAIN. Cạnh (ảnh, contains, khái niệm) của ảnh val/test là chú thích của chính ứng viên, được dùng, nhưng phải ghi rõ hạn chế: thực tế ảnh mới không có scene graph gán tay. ConceptNet là tri thức ngoài, không phụ thuộc split.</t>
+          <t>Đồ thị của ảnh nào chỉ chứa chú thích của chính ảnh đó, không có cạnh gộp qua nhiều ảnh, nên không có thống kê nào của val/test lọt vào huấn luyện; GAT học trên ảnh TRAIN rồi áp lên ảnh val/test như dữ liệu mới. Hạn chế phải ghi rõ: scene graph của ảnh ứng viên là chú thích gán tay, thực tế ảnh mới không có sẵn. Rủi ro: nếu tỉ lệ (c) thấp thì hướng khớp bộ ba không có tác dụng, phải xét lại thiết kế.</t>
         </is>
       </c>
       <c r="H9" s="20" t="inlineStr">
         <is>
-          <t>Bảng thống kê: số node mỗi loại, số cạnh mỗi loại, bậc trung bình, tỉ lệ ảnh không còn đối tượng nào sau lọc.</t>
+          <t>Bảng thống kê: số đối tượng, số quan hệ mỗi ảnh (trung bình, trung vị), tỉ lệ ảnh không còn quan hệ; ba tỉ lệ (a)(b)(c) có số thật trên train/val.</t>
         </is>
       </c>
       <c r="I9" s="20" t="inlineStr">
@@ -1885,38 +1887,38 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Nối truy vấn vào đồ thị</t>
+          <t>Đồ thị truy vấn</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>Caption (truy vấn), danh sách node khái niệm, alias.</t>
+          <t>Caption (truy vấn), alias và nhãn VG150.</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>Tách danh từ và động từ bằng spaCy, lấy lemma, khớp vào tên node khái niệm (qua alias). Kết quả: mỗi truy vấn → tập node khái niệm xuất phát. Truy vấn không khớp node nào thì điểm đồ thị = 0, chỉ còn điểm CLIP.</t>
+          <t>Tách caption thành đồ thị nhỏ cùng dạng với scene graph: đối tượng, quan hệ, bộ ba, ví dụ "a child playing with a ball" → (child, playing with, ball). Dùng bộ tách dựa trên spaCy (SceneGraphParser hoặc luật trên cây phụ thuộc). Chuẩn hoá tên theo alias; từ không có trong VG150 vẫn giữ, vì node mang vector CLIP text nên kid và child tự gần nhau. Truy vấn không tách được bộ ba nào thì khớp ở mức đối tượng; không có đối tượng nào thì điểm đồ thị = 0, chỉ còn điểm CLIP.</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>data/processed/query_concepts_{train,val,test}.json
-thống kê tỉ lệ truy vấn khớp ≥1 node</t>
+          <t>data/processed/query_graphs_{train,val,test}.json
+thống kê tỉ lệ truy vấn tách được ≥1 bộ ba</t>
         </is>
       </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
-          <t>src/graph/link_query.py, spacy (en_core_web_sm)</t>
+          <t>src/graph/parse_query.py, spacy (en_core_web_sm), SceneGraphParser</t>
         </is>
       </c>
       <c r="G10" s="20" t="inlineStr">
         <is>
-          <t>Bước này không học gì nên không rò rỉ. Rủi ro: tỉ lệ khớp thấp thì đồ thị không có tác dụng; nếu dưới ~70% thì mở rộng alias hoặc khớp gần đúng bằng vector CLIP text.</t>
+          <t>Bước này không học gì nên không rò rỉ. Rủi ro lớn nhất của cả cấp độ 1: bộ tách bắt sai hoặc bỏ sót quan hệ thì các bước sau vô nghĩa, nên đo ở bước 1.5 trước khi viết GNN.</t>
         </is>
       </c>
       <c r="H10" s="20" t="inlineStr">
         <is>
-          <t>Tỉ lệ truy vấn khớp ≥1 node được báo cáo cho cả 3 split; xem tay 30 truy vấn để kiểm tra khớp sai.</t>
+          <t>Tỉ lệ truy vấn tách được ≥1 bộ ba và ≥1 đối tượng được báo cáo cho cả 3 split; xem tay 30 truy vấn để kiểm tra tách sai.</t>
         </is>
       </c>
       <c r="I10" s="20" t="inlineStr">
@@ -1938,28 +1940,28 @@
       </c>
       <c r="C11" s="20" t="inlineStr">
         <is>
-          <t>Đồ thị, query_concepts, top-50 của baseline, split train/val.</t>
+          <t>Scene graph từng ảnh, đồ thị truy vấn, top-50 của baseline, split train/val.</t>
         </is>
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
-          <t>GAT 2 lớp trên đồ thị (đa quan hệ: mỗi loại cạnh một bộ trọng số, hoặc nhúng loại cạnh vào attention). Biểu diễn truy vấn = gộp embedding các node khái niệm xuất phát. Điểm đồ thị(truy vấn, ảnh) = cosine giữa biểu diễn truy vấn và embedding GNN của node ảnh. Huấn luyện bằng contrastive loss trên cặp (caption, ảnh) của TRAIN; dừng sớm theo Recall trên VAL. Chạy ≥3 seed.</t>
+          <t>Một GAT 2 lớp dùng chung, chạy trong từng đồ thị nhỏ (cả ảnh lẫn truy vấn), đưa loại quan hệ vào attention. Sau GAT, mỗi bộ ba có một vector (gộp chủ thể, quan hệ, đối tượng). Điểm đồ thị(truy vấn, ảnh) = trung bình, trên các bộ ba của truy vấn, của cosine lớn nhất với một bộ ba của ảnh; cộng thêm mức đối tượng khi truy vấn không có bộ ba. Huấn luyện bằng contrastive loss trên cặp (caption, ảnh) của TRAIN, ảnh âm lấy trong batch và trong top-50 của CLIP; dừng sớm theo Recall trên VAL. Chạy ≥3 seed.</t>
         </is>
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>src/models/gat_ranker.py, src/train.py
+          <t>src/models/graph_matcher.py, src/train.py
 experiments/level1/gat/seed_{0,1,2}/ (checkpoint, log, config)</t>
         </is>
       </c>
       <c r="F11" s="20" t="inlineStr">
         <is>
-          <t>torch_geometric (GATConv / HGTConv), torch</t>
+          <t>torch_geometric (GATConv / GATv2Conv có edge_attr), torch</t>
         </is>
       </c>
       <c r="G11" s="20" t="inlineStr">
         <is>
-          <t>Caption test không bao giờ vào huấn luyện. Thiết kế phải để giải thích sinh từ cơ chế chấm điểm: giữ lại attention từng cạnh và đóng góp của từng node khái niệm vào điểm, không tìm đường đi sau khi đã xếp hạng (đề cấm).</t>
+          <t>Caption test không bao giờ vào huấn luyện. Giải thích sinh từ cơ chế chấm điểm: điểm là tổng đóng góp của từng cặp bộ ba khớp nên giữ lại chính các cặp đó, không tìm đường đi sau khi đã xếp hạng (đề cấm).</t>
         </is>
       </c>
       <c r="H11" s="20" t="inlineStr">
@@ -2033,17 +2035,17 @@
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
-          <t>Đồ thị, pipeline 1.7–1.8.</t>
+          <t>Scene graph từng ảnh, pipeline 1.7–1.8.</t>
         </is>
       </c>
       <c r="D13" s="20" t="inlineStr">
         <is>
-          <t>Huấn luyện lại với: (a) bỏ cạnh quan hệ, chỉ giữ contains; (b) bỏ cạnh ConceptNet; (c) xáo cạnh, giữ nguyên bậc node; (d) đồ thị ngẫu nhiên cùng số cạnh. Cùng seed, cùng siêu tham số với bản đầy đủ.</t>
+          <t>Huấn luyện lại với: (a) bỏ cạnh quan hệ, chỉ còn tập đối tượng; (b) xáo cạnh trong từng scene graph, giữ nguyên tập node và số cạnh; (c) scene graph ngẫu nhiên: gán cho mỗi ảnh đồ thị của một ảnh khác cùng split. Cùng seed, cùng siêu tham số với bản đầy đủ.</t>
         </is>
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>experiments/level1/ablation/{no_rel,no_conceptnet,shuffled,random}/
+          <t>experiments/level1/ablation/{no_rel,shuffled,random}/
 bảng tổng hợp ablation</t>
         </is>
       </c>
@@ -2054,12 +2056,12 @@
       </c>
       <c r="G13" s="20" t="inlineStr">
         <is>
-          <t>Mục đích là chứng minh cải thiện đến từ cấu trúc quan hệ. Nếu (c) và (d) cho kết quả ngang bản đầy đủ thì đồ thị không đóng góp gì: phải báo cáo đúng như vậy, không che.</t>
+          <t>Mục đích là chứng minh cải thiện đến từ cấu trúc quan hệ. Nếu (a) và (b) cho kết quả ngang bản đầy đủ thì quan hệ không đóng góp gì, chỉ có danh sách đối tượng giúp: phải báo cáo đúng như vậy, không che.</t>
         </is>
       </c>
       <c r="H13" s="20" t="inlineStr">
         <is>
-          <t>Bảng 5 hàng (đầy đủ + 4 biến thể) × 4 metric, mean ± std.</t>
+          <t>Bảng 4 hàng (đầy đủ + 3 biến thể) × 4 metric, mean ± std.</t>
         </is>
       </c>
       <c r="I13" s="20" t="inlineStr">
@@ -2081,12 +2083,12 @@
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>Checkpoint GAT, đồ thị, truy vấn.</t>
+          <t>Checkpoint GAT, scene graph, đồ thị truy vấn.</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
         <is>
-          <t>Với mỗi kết quả: lấy các node khái niệm xuất phát của truy vấn, lần theo cạnh có attention cao nhất tới node ảnh, xuất top-m đường đi kèm trọng số đóng góp vào điểm đồ thị. Trả về cấu trúc dữ liệu (danh sách đường đi + trọng số) để platform demo ở bước 1.12 hiển thị.</t>
+          <t>Với mỗi kết quả: xuất top-m cặp (bộ ba của truy vấn ↔ bộ ba của ảnh) khớp cao nhất kèm đóng góp vào điểm đồ thị, ví dụ (child, playing with, ball) ↔ (child –holding→ ball): 0,41. Trả về cấu trúc dữ liệu (danh sách cạnh + trọng số) để platform demo ở bước 1.12 hiển thị.</t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">
@@ -2102,12 +2104,12 @@
       </c>
       <c r="G14" s="20" t="inlineStr">
         <is>
-          <t>Đường đi hiển thị phải là thứ thật sự tham gia tính điểm. Thiết kế sẵn hàm "bỏ các cạnh này rồi tính lại điểm" vì cấp độ 3 đo fidelity bằng đúng hàm đó.</t>
+          <t>Thứ hiển thị phải là thứ thật sự tham gia tính điểm. Thiết kế sẵn hàm "bỏ các bộ ba này khỏi scene graph rồi tính lại điểm" vì cấp độ 3 đo fidelity bằng đúng hàm đó.</t>
         </is>
       </c>
       <c r="H14" s="20" t="inlineStr">
         <is>
-          <t>Hàm giải thích có test; mỗi kết quả có ≥1 đường đi hoặc ghi rõ "không có đường đi, chỉ dùng điểm CLIP".</t>
+          <t>Hàm giải thích có test; mỗi kết quả có ≥1 cặp bộ ba khớp hoặc ghi rõ "không có bộ ba khớp, chỉ dùng điểm CLIP".</t>
         </is>
       </c>
       <c r="I14" s="20" t="inlineStr">
@@ -2233,10 +2235,10 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
+    <row r="21" ht="60" customHeight="1">
       <c r="A21" s="22" t="inlineStr">
         <is>
-          <t>3. Cách biểu diễn quan hệ trong scene graph: cạnh gộp khái niệm–khái niệm (đơn giản, mất thông tin "quan hệ này ở ảnh nào") hay thêm node bộ ba nối với ảnh (giữ được, đồ thị lớn hơn). Đề xuất bắt đầu bằng cách gộp, thêm node bộ ba nếu ablation cho thấy cạnh quan hệ không giúp gì.</t>
+          <t>3. Cách dùng scene graph: ĐỔI 2026-09-19. Bỏ phương án một đồ thị chung (node ảnh + node khái niệm + cạnh ConceptNet); dùng đồ thị riêng từng ảnh so với đồ thị tách từ truy vấn, khớp ở mức bộ ba. Lý do: đây là hướng của đa số bài đã công bố (SGM, GSMN, SEMScene, CORA), giữ được "quan hệ này ở ảnh nào", không rò rỉ vì không có cạnh gộp qua ảnh, và giải thích đến thẳng từ điểm. Khảo sát: docs/research/graph-enhanced-image-retrieval-approaches.md. Thiết kế còn phụ thuộc số đo ở bước 1.5; nếu tỉ lệ bộ ba khớp quá thấp thì xét lại.</t>
         </is>
       </c>
     </row>
@@ -2261,8 +2263,16 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>7. ConceptNet không dùng ở cấp độ 1. Thêm ở cấp độ 2 như một lớp khái niệm nhỏ (không có node ảnh) cho truy vấn gián tiếp, bật/tắt để đo đóng góp.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="A25:I25"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
docs: assign graph building task to Loc
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -844,14 +844,18 @@
           <t>Visual Genome ∩ COCO</t>
         </is>
       </c>
-      <c r="D12" s="7" t="n"/>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="7" t="n"/>
       <c r="G12" s="7" t="n"/>
       <c r="H12" s="7" t="n"/>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: mark Loc on level 1 query graph, GAT, rerank, ablation and explanation tasks
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phan cong" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cap do 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Phan cong" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cap do 1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -871,14 +871,18 @@
           <t>Visual Genome ∩ COCO</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n"/>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="7" t="n"/>
       <c r="G13" s="7" t="n"/>
       <c r="H13" s="7" t="n"/>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>
@@ -894,14 +898,18 @@
           <t>Visual Genome ∩ COCO</t>
         </is>
       </c>
-      <c r="D14" s="7" t="n"/>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="7" t="n"/>
       <c r="G14" s="7" t="n"/>
       <c r="H14" s="7" t="n"/>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>
@@ -917,14 +925,18 @@
           <t>Visual Genome ∩ COCO</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n"/>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="E15" s="7" t="n"/>
       <c r="F15" s="7" t="n"/>
       <c r="G15" s="7" t="n"/>
       <c r="H15" s="7" t="n"/>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>
@@ -940,14 +952,18 @@
           <t>Visual Genome ∩ COCO</t>
         </is>
       </c>
-      <c r="D16" s="7" t="n"/>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="7" t="n"/>
       <c r="H16" s="7" t="n"/>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>
@@ -963,14 +979,18 @@
           <t>Visual Genome ∩ COCO</t>
         </is>
       </c>
-      <c r="D17" s="7" t="n"/>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
       <c r="G17" s="7" t="n"/>
       <c r="H17" s="7" t="n"/>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(level2): NativE reproduction setup notes, MKG-W data audit and CPU smoke test
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -771,16 +771,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -836,7 +840,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -852,7 +856,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1115,734 +1119,734 @@
   <dimension ref="A1:I41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7" t="s">
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="6" t="s">
+      <c r="A7" s="6"/>
+      <c r="B7" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7" t="s">
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6" t="s">
+      <c r="A8" s="6"/>
+      <c r="B8" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7" t="s">
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6" t="s">
+      <c r="A9" s="6"/>
+      <c r="B9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7" t="s">
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7" t="s">
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8"/>
-      <c r="B11" s="9" t="s">
+      <c r="A11" s="9"/>
+      <c r="B11" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7" t="s">
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8"/>
-      <c r="B12" s="9" t="s">
+      <c r="A12" s="9"/>
+      <c r="B12" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7" t="s">
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8"/>
-      <c r="B13" s="9" t="s">
+      <c r="A13" s="9"/>
+      <c r="B13" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7" t="s">
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8"/>
-      <c r="B14" s="9" t="s">
+      <c r="A14" s="9"/>
+      <c r="B14" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7" t="s">
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8"/>
-      <c r="B15" s="9" t="s">
+      <c r="A15" s="9"/>
+      <c r="B15" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7" t="s">
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8"/>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="9"/>
+      <c r="B16" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7" t="s">
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8"/>
-      <c r="B17" s="9" t="s">
+      <c r="A17" s="9"/>
+      <c r="B17" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7" t="s">
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8"/>
-      <c r="B18" s="9" t="s">
+      <c r="A18" s="9"/>
+      <c r="B18" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7" t="s">
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8"/>
-      <c r="B19" s="9" t="s">
+      <c r="A19" s="9"/>
+      <c r="B19" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="7" t="s">
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7" t="s">
+      <c r="D20" s="8"/>
+      <c r="E20" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="7" t="s">
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10"/>
-      <c r="B21" s="11" t="s">
+      <c r="A21" s="11"/>
+      <c r="B21" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7" t="s">
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10"/>
-      <c r="B22" s="11" t="s">
+      <c r="A22" s="11"/>
+      <c r="B22" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7" t="s">
+      <c r="D22" s="8"/>
+      <c r="E22" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7" t="s">
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11"/>
+      <c r="B23" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10"/>
-      <c r="B23" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7" t="s">
+    <row r="24" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11"/>
+      <c r="B24" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11"/>
+      <c r="B25" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11"/>
+      <c r="B26" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7" t="s">
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10"/>
-      <c r="B24" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="11" t="s">
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13"/>
+      <c r="B28" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7" t="s">
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10"/>
-      <c r="B25" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="C25" s="11" t="s">
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="13"/>
+      <c r="B29" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="C29" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7" t="s">
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10"/>
-      <c r="B26" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="C26" s="11" t="s">
+    <row r="30" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="13"/>
+      <c r="B30" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="13"/>
+      <c r="B31" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13"/>
+      <c r="B32" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8"/>
+      <c r="I32" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C33" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7" t="s">
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="C27" s="13" t="s">
+    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="15"/>
+      <c r="B34" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7" t="s">
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12"/>
-      <c r="B28" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7" t="s">
+    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12"/>
-      <c r="B29" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
-      <c r="H29" s="7"/>
-      <c r="I29" s="7" t="s">
+    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6"/>
+      <c r="B36" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="12"/>
-      <c r="B30" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
-      <c r="G30" s="7"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="7" t="s">
+    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6"/>
+      <c r="B37" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12"/>
-      <c r="B31" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C31" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7" t="s">
+    <row r="38" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6"/>
+      <c r="B38" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="12"/>
-      <c r="B32" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B33" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="14"/>
-      <c r="B34" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="C34" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5"/>
-      <c r="B36" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5"/>
-      <c r="B37" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5"/>
-      <c r="B38" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="E38" s="7"/>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C40" s="16" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C40" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="D40" s="17" t="n">
+      <c r="D40" s="18" t="n">
         <f aca="false">COUNTIF(D6:D38,"Chính")</f>
         <v>12</v>
       </c>
-      <c r="E40" s="17" t="n">
+      <c r="E40" s="18" t="n">
         <f aca="false">COUNTIF(E6:E38,"Chính")</f>
         <v>4</v>
       </c>
-      <c r="F40" s="17" t="n">
+      <c r="F40" s="18" t="n">
         <f aca="false">COUNTIF(F6:F38,"Chính")</f>
         <v>0</v>
       </c>
-      <c r="G40" s="17" t="n">
+      <c r="G40" s="18" t="n">
         <f aca="false">COUNTIF(G6:G38,"Chính")</f>
         <v>0</v>
       </c>
-      <c r="H40" s="17" t="n">
+      <c r="H40" s="18" t="n">
         <f aca="false">COUNTIF(H6:H38,"Chính")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C41" s="16" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C41" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="D41" s="17" t="n">
+      <c r="D41" s="18" t="n">
         <f aca="false">COUNTIF(D6:D38,"Hỗ trợ")</f>
         <v>1</v>
       </c>
-      <c r="E41" s="17" t="n">
+      <c r="E41" s="18" t="n">
         <f aca="false">COUNTIF(E6:E38,"Hỗ trợ")</f>
         <v>0</v>
       </c>
-      <c r="F41" s="17" t="n">
+      <c r="F41" s="18" t="n">
         <f aca="false">COUNTIF(F6:F38,"Hỗ trợ")</f>
         <v>0</v>
       </c>
-      <c r="G41" s="17" t="n">
+      <c r="G41" s="18" t="n">
         <f aca="false">COUNTIF(G6:G38,"Hỗ trợ")</f>
         <v>0</v>
       </c>
-      <c r="H41" s="17" t="n">
+      <c r="H41" s="18" t="n">
         <f aca="false">COUNTIF(H6:H38,"Hỗ trợ")</f>
         <v>0</v>
       </c>
@@ -1887,515 +1891,515 @@
   <dimension ref="A1:I25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="5" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="I5" s="19" t="s">
+      <c r="I5" s="20" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="I6" s="19" t="s">
+      <c r="I6" s="20" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="H7" s="19" t="s">
+      <c r="H7" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="I7" s="19" t="s">
+      <c r="I7" s="20" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="20" t="s">
         <v>109</v>
       </c>
-      <c r="I8" s="19" t="s">
+      <c r="I8" s="20" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="G9" s="15" t="s">
+      <c r="G9" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="I9" s="19" t="s">
+      <c r="I9" s="20" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="H10" s="19" t="s">
+      <c r="H10" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="I10" s="19" t="s">
+      <c r="I10" s="20" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="H11" s="19" t="s">
+      <c r="H11" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="I11" s="19" t="s">
+      <c r="I11" s="20" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="20" t="s">
         <v>138</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H12" s="19" t="s">
+      <c r="H12" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="I12" s="19" t="s">
+      <c r="I12" s="20" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>145</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="20" t="s">
         <v>146</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="20" t="s">
         <v>147</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="20" t="s">
         <v>150</v>
       </c>
-      <c r="H13" s="19" t="s">
+      <c r="H13" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="I13" s="19" t="s">
+      <c r="I13" s="20" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>153</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="20" t="s">
         <v>156</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="H14" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="I14" s="19" t="s">
+      <c r="I14" s="20" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="F15" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="G15" s="20" t="s">
         <v>166</v>
       </c>
-      <c r="H15" s="19" t="s">
+      <c r="H15" s="20" t="s">
         <v>167</v>
       </c>
-      <c r="I15" s="19" t="s">
+      <c r="I15" s="20" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="20" t="s">
         <v>170</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="20" t="s">
         <v>172</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="G16" s="20" t="s">
         <v>174</v>
       </c>
-      <c r="H16" s="19" t="s">
+      <c r="H16" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="I16" s="19" t="s">
+      <c r="I16" s="20" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="22" t="s">
         <v>178</v>
       </c>
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="21"/>
-      <c r="H19" s="21"/>
-      <c r="I19" s="21"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="22" t="s">
         <v>179</v>
       </c>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="21"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
     </row>
     <row r="21" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="22" t="s">
         <v>180</v>
       </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="21"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="22" t="s">
         <v>181</v>
       </c>
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="21"/>
-      <c r="I22" s="21"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="22"/>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="22" t="s">
         <v>182</v>
       </c>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="21"/>
-      <c r="I23" s="21"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
+      <c r="I23" s="22"/>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="B24" s="21"/>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="21"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+      <c r="I24" s="22"/>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="22" t="s">
         <v>184</v>
       </c>
-      <c r="B25" s="21"/>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
docs: Nhi claims xAI evaluation tasks (fidelity, validity, sparsity)
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -1160,7 +1160,11 @@
       <c r="D27" s="12" t="n"/>
       <c r="E27" s="12" t="n"/>
       <c r="F27" s="12" t="n"/>
-      <c r="G27" s="12" t="n"/>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="H27" s="12" t="n"/>
       <c r="I27" s="12" t="inlineStr">
         <is>
@@ -1183,7 +1187,11 @@
       <c r="D28" s="12" t="n"/>
       <c r="E28" s="12" t="n"/>
       <c r="F28" s="12" t="n"/>
-      <c r="G28" s="12" t="n"/>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="H28" s="12" t="n"/>
       <c r="I28" s="12" t="inlineStr">
         <is>
@@ -1206,7 +1214,11 @@
       <c r="D29" s="12" t="n"/>
       <c r="E29" s="12" t="n"/>
       <c r="F29" s="12" t="n"/>
-      <c r="G29" s="12" t="n"/>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="H29" s="12" t="n"/>
       <c r="I29" s="12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: Nhi claims the VG-COCO evaluation query set (row 24)
</commit_message>
<xml_diff>
--- a/task-assignment.xlsx
+++ b/task-assignment.xlsx
@@ -1083,7 +1083,11 @@
       <c r="D24" s="12" t="n"/>
       <c r="E24" s="12" t="n"/>
       <c r="F24" s="12" t="n"/>
-      <c r="G24" s="12" t="n"/>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>Chính</t>
+        </is>
+      </c>
       <c r="H24" s="12" t="n"/>
       <c r="I24" s="12" t="inlineStr">
         <is>

</xml_diff>